<commit_message>
Add pooled repetition mode, avatar views, and 671/252 exploration pipeline.
Skeleton conversion now falls back through sidecar and raw hierarchy resolution; validation scores all longitudinal comparisons against NV; UI gains Avatar Views tab and repetition-mode controls.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/segmentation/252_ex_segmentatios_frames.xlsx
+++ b/data/segmentation/252_ex_segmentatios_frames.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/drorhazan/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/drorhazan/Desktop/gaga_psilo/projects/gaga_jcvpca/data/segmentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C0CF93E-92A4-6548-A0C0-0ABA59F3248C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4B6EF80-8C48-1C40-A726-AF648E115611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="5" xr2:uid="{5B81ED3C-114E-4DB1-B102-58D9FAB272D1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="5" xr2:uid="{5B81ED3C-114E-4DB1-B102-58D9FAB272D1}"/>
   </bookViews>
   <sheets>
     <sheet name="252 - T1P1R1" sheetId="1" r:id="rId1"/>
@@ -3060,7 +3060,7 @@
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.5" customWidth="1"/>
+    <col min="2" max="2" width="39" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>